<commit_message>
Update issue tracker overview spreadsheet
Refresh the Megalijst issue tracker overview workbook with the latest project data. This change updates the spreadsheet contents used to track and review issue status and summary information.
</commit_message>
<xml_diff>
--- a/Megalijst/issue-tracker-overzicht.xlsx
+++ b/Megalijst/issue-tracker-overzicht.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1163" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1173" uniqueCount="533">
   <si>
     <t>Fase</t>
   </si>
@@ -1511,6 +1511,135 @@
   </si>
   <si>
     <t>Jira-status = Special action; Baas mondeling/schriftelijk beschikbaar; Mail met beschrijving speciale actie; Goedkeuring; Jira-uitvoerder wordt de baas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analysing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analysing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Review Analyse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Review Analyse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Designing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Designing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Review design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Review design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SpecialAction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SpecialAction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volg de review ontwerp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eindevent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naar flowchartpagina review ontwerp navigeren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volg de meldplicht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eindevent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naar flowchartpagina meldplicht navigeren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volg de test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eindevent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naar flowchartpagina test navigeren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volg de meldplicht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eindevent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naar flowchartpagina meldplicht navigeren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jira-status = SpecialAction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jira-uitvoerder = medewerker; Jira-status = SpecialAction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jira-status wordt Analysing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jira-status wordt Designing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jira-status wordt Implementing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jira-status wordt Testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actiecode(s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bron</t>
+  </si>
+  <si>
+    <t xml:space="preserve">102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Issue Tracker intake.drawio#diagram=_NZFfUYCCha4VbYokAiz;kind=node;id=bpmn_task_oplossingsrichting;Action=102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Issue Tracker intake.drawio#diagram=_NZFfUYCCha4VbYokAiz;kind=node;id=bpmn_task_deliverables;Action=103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 Issue Tracker review final.drawio#diagram=mpQzUtWff58q1bPTKcpG-1;kind=node;id=bpmn_task_intake;Action=1003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 Issue Tracker review final.drawio#diagram=mpQzUtWff58q1bPTKcpG-1;kind=node;id=bpmn_task_beoordeling;Action=1005</t>
   </si>
 </sst>
 </file>
@@ -2172,7 +2301,7 @@
         <v>9</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>12</v>
+        <v>490</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>14</v>
@@ -2186,10 +2315,10 @@
         <v>16</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>12</v>
+        <v>491</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>15</v>
+        <v>492</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>17</v>
@@ -2203,10 +2332,10 @@
         <v>19</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>15</v>
+        <v>493</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>18</v>
+        <v>494</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>20</v>
@@ -2220,10 +2349,10 @@
         <v>22</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>18</v>
+        <v>495</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>21</v>
+        <v>496</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>23</v>
@@ -2237,10 +2366,10 @@
         <v>25</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>21</v>
+        <v>497</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>24</v>
+        <v>498</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>26</v>
@@ -2254,10 +2383,10 @@
         <v>28</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>24</v>
+        <v>499</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>27</v>
+        <v>500</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>29</v>
@@ -2271,10 +2400,10 @@
         <v>31</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>27</v>
+        <v>501</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>32</v>
+        <v>502</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>33</v>
@@ -2305,10 +2434,10 @@
         <v>40</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>41</v>
+        <v>503</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>42</v>
+        <v>504</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>43</v>
@@ -3072,13 +3201,13 @@
         <v>18</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>70</v>
+        <v>505</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>71</v>
+        <v>506</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>72</v>
+        <v>507</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3089,13 +3218,13 @@
         <v>18</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>155</v>
+        <v>508</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>71</v>
+        <v>509</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>75</v>
+        <v>510</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3480,13 +3609,13 @@
         <v>24</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>70</v>
+        <v>511</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>71</v>
+        <v>512</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>72</v>
+        <v>513</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3497,13 +3626,13 @@
         <v>24</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>193</v>
+        <v>514</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>71</v>
+        <v>515</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>75</v>
+        <v>516</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -4183,7 +4312,7 @@
         <v>141</v>
       </c>
       <c r="E107" s="3" t="s">
-        <v>273</v>
+        <v>517</v>
       </c>
     </row>
     <row r="108" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -4489,7 +4618,7 @@
         <v>141</v>
       </c>
       <c r="E125" s="3" t="s">
-        <v>302</v>
+        <v>518</v>
       </c>
     </row>
     <row r="126" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -4623,7 +4752,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E110"/>
+  <dimension ref="A1:G110"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -4649,6 +4778,12 @@
       <c r="E1" s="1" t="s">
         <v>314</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>524</v>
+      </c>
     </row>
     <row r="2" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
@@ -4754,6 +4889,12 @@
         <v>335</v>
       </c>
       <c r="E8" s="3"/>
+      <c r="F8" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>526</v>
+      </c>
     </row>
     <row r="9" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -4769,6 +4910,12 @@
         <v>338</v>
       </c>
       <c r="E9" s="3"/>
+      <c r="F9" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>528</v>
+      </c>
     </row>
     <row r="10" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
@@ -5063,7 +5210,7 @@
         <v>12</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>376</v>
+        <v>519</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>323</v>
@@ -5489,7 +5636,7 @@
         <v>18</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>405</v>
+        <v>520</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>323</v>
@@ -5868,7 +6015,7 @@
         <v>24</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>434</v>
+        <v>521</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>323</v>
@@ -6054,7 +6201,7 @@
         <v>27</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>457</v>
+        <v>522</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>323</v>
@@ -6263,6 +6410,12 @@
         <v>482</v>
       </c>
       <c r="E107" s="3"/>
+      <c r="F107" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="G107" s="3" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="108" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A108" s="3" t="s">
@@ -6278,6 +6431,12 @@
         <v>483</v>
       </c>
       <c r="E108" s="3"/>
+      <c r="F108" s="3" t="s">
+        <v>531</v>
+      </c>
+      <c r="G108" s="3" t="s">
+        <v>532</v>
+      </c>
     </row>
     <row r="109" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" s="3" t="s">
@@ -6310,7 +6469,7 @@
       <c r="E110" s="3"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:E110">
+  <conditionalFormatting sqref="A2:G110">
     <cfRule type="expression" dxfId="11" priority="2">
       <formula>$B2="Intake"</formula>
     </cfRule>

</xml_diff>